<commit_message>
Fix watchlist sync source
</commit_message>
<xml_diff>
--- a/watch_list.xlsx
+++ b/watch_list.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>股票名称</t>
   </si>
@@ -78,6 +78,15 @@
   </si>
   <si>
     <t>300499</t>
+  </si>
+  <si>
+    <t>数据港</t>
+  </si>
+  <si>
+    <t>603881</t>
+  </si>
+  <si>
+    <t>数据中心</t>
   </si>
 </sst>
 </file>
@@ -1225,8 +1234,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="2"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="13.6153846153846" customWidth="1"/>
     <col min="2" max="2" width="13.1346153846154" customWidth="1"/>
@@ -1309,6 +1318,17 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>